<commit_message>
DEGS1-1 DD and DPE with additional variables for P1
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_dictionary/DD_DEGS1_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_dictionary/DD_DEGS1_FRANZI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Projekte\NFDI4Health\TA5\Pilotprojekte\Harmonisierung\HarmonizR\use-cases-harmonisation\analyst\Franzi\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E9ED5FD0-1232-4A8E-9BEE-23955EEB5D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848F514D-B7F3-4040-86AB-93DB993F809C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43305" yWindow="2205" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="136">
   <si>
     <t>index</t>
   </si>
@@ -367,6 +367,84 @@
   </si>
   <si>
     <t>Kartoffelchips g/Tag</t>
+  </si>
+  <si>
+    <t>sex</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>SDisced97z</t>
+  </si>
+  <si>
+    <t>RCstat_k</t>
+  </si>
+  <si>
+    <t>Usbmi</t>
+  </si>
+  <si>
+    <t>ISCED (1997) - Klassifikation</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>Alter (in vollendeten Lebensjahren)</t>
+  </si>
+  <si>
+    <t>Geschlecht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">integer </t>
+  </si>
+  <si>
+    <t>Rauchstatus in 3 Kategorien</t>
+  </si>
+  <si>
+    <t>Body-Mass-Index [kg/m2]</t>
+  </si>
+  <si>
+    <t>männlich</t>
+  </si>
+  <si>
+    <t>weiblich</t>
+  </si>
+  <si>
+    <t>3b</t>
+  </si>
+  <si>
+    <t>3A</t>
+  </si>
+  <si>
+    <t>4A</t>
+  </si>
+  <si>
+    <t>5B</t>
+  </si>
+  <si>
+    <t>5A</t>
+  </si>
+  <si>
+    <t>(Gelegenheits-)Raucher</t>
+  </si>
+  <si>
+    <t>Exraucher</t>
+  </si>
+  <si>
+    <t>Nieraucher</t>
+  </si>
+  <si>
+    <t>missing</t>
+  </si>
+  <si>
+    <t>Filterbed. Fehlend (lebt nicht in HH)</t>
+  </si>
+  <si>
+    <t>Nicht erhoben (18+ Jahre)</t>
+  </si>
+  <si>
+    <t>Nicht erhoben</t>
   </si>
 </sst>
 </file>
@@ -423,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -433,6 +511,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -737,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -758,56 +839,56 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>6</v>
+        <v>110</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>7</v>
+        <v>118</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>9</v>
+        <v>117</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>113</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>12</v>
+        <v>120</v>
       </c>
       <c r="D5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -815,21 +896,21 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>19</v>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -837,10 +918,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
@@ -848,10 +929,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -859,10 +940,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -870,10 +951,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
@@ -881,10 +962,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -892,10 +973,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -903,10 +984,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>33</v>
+        <v>22</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>23</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -914,10 +995,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>35</v>
+        <v>24</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -925,10 +1006,10 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -936,10 +1017,10 @@
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -947,10 +1028,10 @@
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
@@ -958,10 +1039,10 @@
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>42</v>
+        <v>32</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -969,10 +1050,10 @@
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>45</v>
+        <v>34</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -980,10 +1061,10 @@
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -991,87 +1072,87 @@
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D23" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="3" t="s">
+      <c r="D28" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D24" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="5" t="s">
+      <c r="D29" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="D25" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D28" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D29" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="D30" t="s">
         <v>5</v>
@@ -1079,21 +1160,21 @@
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="5" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>67</v>
+      <c r="B32" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="D32" t="s">
         <v>5</v>
@@ -1101,10 +1182,10 @@
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="D33" t="s">
         <v>5</v>
@@ -1112,21 +1193,21 @@
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D34" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>73</v>
+      <c r="B35" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="D35" t="s">
         <v>5</v>
@@ -1134,10 +1215,10 @@
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D36" t="s">
         <v>5</v>
@@ -1145,10 +1226,10 @@
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D37" t="s">
         <v>5</v>
@@ -1156,10 +1237,10 @@
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="5" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="D38" t="s">
         <v>5</v>
@@ -1167,10 +1248,10 @@
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="5" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
         <v>5</v>
@@ -1178,21 +1259,21 @@
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="5" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="D40" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="2" t="s">
-        <v>84</v>
+      <c r="B41" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D41" t="s">
         <v>5</v>
@@ -1200,10 +1281,10 @@
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
@@ -1211,10 +1292,10 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="5" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D43" t="s">
         <v>5</v>
@@ -1222,10 +1303,10 @@
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="5" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D44" t="s">
         <v>5</v>
@@ -1233,39 +1314,43 @@
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="5" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B46" s="5" t="s">
-        <v>94</v>
+      <c r="B46" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="D46" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="D47" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B48" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>97</v>
+      <c r="B48" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="D48" t="s">
         <v>5</v>
@@ -1273,10 +1358,10 @@
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="5" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D49" t="s">
         <v>5</v>
@@ -1284,43 +1369,39 @@
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>101</v>
+        <v>92</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="D50" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B51" s="3" t="s">
-        <v>102</v>
+      <c r="B51" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D51" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B52" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>105</v>
-      </c>
+    <row r="52" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
       <c r="D52" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B53" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>107</v>
+      <c r="B53" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>97</v>
       </c>
       <c r="D53" t="s">
         <v>5</v>
@@ -1328,12 +1409,67 @@
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B54" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D54" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B55" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D55" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B56" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D56" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B57" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D57" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B58" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D58" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B59" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C54" s="4" t="s">
+      <c r="C59" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D59" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1345,10 +1481,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1357,6 +1497,233 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2">
+        <v>-97</v>
+      </c>
+      <c r="C2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5">
+        <v>-96</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6">
+        <v>-97</v>
+      </c>
+      <c r="C6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2</v>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13">
+        <v>7</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14">
+        <v>8</v>
+      </c>
+      <c r="C14" s="7">
+        <v>6</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>130</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DEGS1-5: finalising DEGS1 documents for harmonisation
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_dictionary/DD_DEGS1_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_dictionary/DD_DEGS1_FRANZI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Franzi\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34790C48-CDE4-466E-944D-6E5377DE2209}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337DBD7C-E095-4936-B627-467DA81DB212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="113">
   <si>
     <t>index</t>
   </si>
@@ -358,50 +358,20 @@
     <t>Kartoffelchips g/Tag</t>
   </si>
   <si>
-    <t>sex</t>
-  </si>
-  <si>
-    <t>age</t>
-  </si>
-  <si>
-    <t>SDisced97z</t>
-  </si>
-  <si>
-    <t>RCstat_k</t>
-  </si>
-  <si>
-    <t>ISCED (1997) - Klassifikation</t>
-  </si>
-  <si>
-    <t>integer</t>
-  </si>
-  <si>
-    <t>Alter (in vollendeten Lebensjahren)</t>
-  </si>
-  <si>
-    <t>Geschlecht</t>
-  </si>
-  <si>
-    <t xml:space="preserve">integer </t>
-  </si>
-  <si>
-    <t>Rauchstatus in 3 Kategorien</t>
-  </si>
-  <si>
     <t>missing</t>
   </si>
   <si>
     <t>mafbier</t>
   </si>
   <si>
-    <t>SOMETHING</t>
+    <t>alkoholfreies Bier ml/Tag</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,14 +396,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -469,7 +431,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -488,9 +450,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -528,9 +490,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -563,26 +525,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -615,26 +560,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -808,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -829,67 +757,67 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
-        <v>110</v>
+        <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>117</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
-        <v>111</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>116</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>112</v>
+        <v>10</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>114</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>113</v>
+        <v>13</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>119</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>8</v>
+      <c r="B7" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
@@ -897,10 +825,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -908,10 +836,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
@@ -919,10 +847,10 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -930,10 +858,10 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -941,10 +869,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
@@ -952,10 +880,10 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -963,10 +891,10 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -974,10 +902,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>25</v>
+        <v>32</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -985,10 +913,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>27</v>
+        <v>34</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -996,10 +924,10 @@
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -1007,10 +935,10 @@
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1018,10 +946,10 @@
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>33</v>
+        <v>41</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
@@ -1029,10 +957,10 @@
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>35</v>
+        <v>43</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -1040,10 +968,10 @@
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -1051,10 +979,10 @@
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -1062,65 +990,65 @@
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>42</v>
+      <c r="B24" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="D24" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>44</v>
+      <c r="B25" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="D25" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="4" t="s">
-        <v>46</v>
+      <c r="B26" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D26" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>48</v>
+      <c r="B27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="D27" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>51</v>
+      <c r="B28" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="D28" t="s">
         <v>5</v>
@@ -1128,32 +1056,32 @@
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D29" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>55</v>
+      <c r="B30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="D30" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>57</v>
+      <c r="B31" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>65</v>
       </c>
       <c r="D31" t="s">
         <v>5</v>
@@ -1161,10 +1089,10 @@
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>59</v>
+        <v>66</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>67</v>
       </c>
       <c r="D32" t="s">
         <v>5</v>
@@ -1172,21 +1100,21 @@
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="5" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>62</v>
+      <c r="B34" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>70</v>
       </c>
       <c r="D34" t="s">
         <v>5</v>
@@ -1194,10 +1122,10 @@
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="5" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="D35" t="s">
         <v>5</v>
@@ -1205,10 +1133,10 @@
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="5" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D36" t="s">
         <v>5</v>
@@ -1216,10 +1144,10 @@
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="5" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D37" t="s">
         <v>5</v>
@@ -1227,10 +1155,10 @@
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="D38" t="s">
         <v>5</v>
@@ -1238,10 +1166,10 @@
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="5" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="D39" t="s">
         <v>5</v>
@@ -1249,21 +1177,21 @@
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="5" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D40" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="5" t="s">
-        <v>76</v>
+      <c r="B41" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="D41" t="s">
         <v>5</v>
@@ -1271,10 +1199,10 @@
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
@@ -1282,10 +1210,10 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="5" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D43" t="s">
         <v>5</v>
@@ -1293,21 +1221,21 @@
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="5" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D44" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B45" s="2" t="s">
-        <v>84</v>
+      <c r="B45" s="5" t="s">
+        <v>92</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
@@ -1315,21 +1243,21 @@
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="5" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="D46" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B47" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>88</v>
+      <c r="B47" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>97</v>
       </c>
       <c r="D47" t="s">
         <v>5</v>
@@ -1337,10 +1265,10 @@
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" s="5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="D48" t="s">
         <v>5</v>
@@ -1348,32 +1276,32 @@
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>93</v>
+        <v>100</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="D49" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B50" s="5" t="s">
-        <v>94</v>
+      <c r="B50" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="D50" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B51" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>97</v>
+      <c r="B51" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="D51" t="s">
         <v>5</v>
@@ -1381,10 +1309,10 @@
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B52" s="5" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="D52" t="s">
         <v>5</v>
@@ -1392,67 +1320,23 @@
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>101</v>
+        <v>108</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="D53" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B54" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>103</v>
+      <c r="B54" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>112</v>
       </c>
       <c r="D54" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B55" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D55" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B56" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D56" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B57" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D57" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B58" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D58" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1482,7 +1366,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>